<commit_message>
Schedule defects sheet: merge C29945 rows, split into Defects-to-file / Reference tabs
Refine the Schedule per-project defect workbook (2026-08-20) for owning QA Ayesha:
- Merge the two C29945 Priority-filter rows into one DO-NOT-FILE reference row
  (Branko ruled it out 19 Aug 2026, latest authoritative word per Standing Rule 32;
  note preserves the earlier 'deferred' history; keeps C29945/C29942 + both sources).
- Split the single Defects tab into 'Defects to file' (4 actionable create-new/reopen
  rows) and 'Reference - do not file' (7 informational rows incl. the merged C29945).
- Update Summary tab with the split, owning QA, date, and 12->11 reconciliation.
- Regenerate .xlsx (real newlines, wrapped) and .md twin (<br>). Report Suite and
  Filters sheets untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/schedule/build-verify-2026-08-18/Schedule_Defects-for-Testers_2026-08-20.xlsx
+++ b/build/schedule/build-verify-2026-08-18/Schedule_Defects-for-Testers_2026-08-20.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Defects" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Defects to file" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Reference - do not file" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,25 +61,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D0D0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,10 +74,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -458,11 +442,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,56 +483,102 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Defect rows</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>12</v>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
+          <t>Rows (pre-merge)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Schedule defects for the manual tester to review and file as Jira Story Defects (create-new, reopen, and not-defect rows are marked in the last column).</t>
-        </is>
+          <t>Rows (post-merge, distinct)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Split</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Split from the combined Report Suite + Schedule Defects-for-Testers sheet (2026-08-19) plus project-specific build-verify findings; build v3.8.</t>
+          <t>4 defects to file / 7 reference rows (do not file)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Defects to file</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>4 — the genuinely actionable Story Defects Ayesha should raise (create-new + reopen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Reference - do not file</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>7 — informational only: not-a-defect, feature-not-built, ruled-out, and automation-held rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Merge note</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>The two Priority-filter rows for case C29945 were merged into ONE reference row; this reduced the total from 12 to 11 distinct rows. Branko ruled the Priority filter out of scope on 19 Aug 2026, so the merged row is DO NOT FILE (its note preserves the earlier 'deferred' history).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Schedule defects for the manual tester (Ayesha) to review. The 'Defects to file' tab lists what to raise as Jira Story Defects; the 'Reference - do not file' tab is informational only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Expected behavior comes from the documented source (spec / epic / PO answer), never the build (Standing Rule 57). Jira ticket creation is on hold — this sheet is for the manual QA to read and then create the Story Defects.</t>
         </is>
@@ -565,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -627,121 +657,72 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Sidebar - Work Order Filters</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Priority filter group missing from the sidebar Filters panel</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>The sidebar Filters popup contains only Assignment (Unassigned/Assigned) and Status; there is no Priority group (High/Medium/Low). Confirmed by reading the full popup and a body-wide search.</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>1. Open Schedule.
-2. Click the sidebar Filters button.
-3. Look for a Priority group with High / Medium / Low options.</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>The Filters panel offers three groups: Assignment, Status, and Priority (High, Medium, Low).</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Schedule specification v30 §5.1 / story SV-8687; epic SV-8685.</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>C29945</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29945</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Recommendation: DEFERRED (feature not found — confirm with Branko whether Priority filtering is in V1; re-check when it ships). Existing ticket: NO TICKET (feature not found — Rule 69 deferred). Reproduces on v3.8-bd246fd: Yes (Priority group absent on v3.8-bd246fd).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Conflict Detection</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Conflict shifts are styled amber, not red</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>A double-booked (conflicted) shift is highlighted with an amber warning colour and an amber warning icon. The specification says red styling is reserved for conflicts and errors, so a conflict should read as red, not amber.</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Find a technician who has two overlapping shifts on the same day (a double-booked / conflict shift — the board already has some, e.g. around Aug 26).
 3. Look at the conflict shift block and its warning icon and note the colour.</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Conflicts (and errors) are shown in RED. Red styling is reserved for conflicts and errors, and is never used for overtime.</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.11 (styling rule) / §4.12; story SV-8697; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>C30029</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/30029</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Category: CREATE NEW. Recommended action: CREATE NEW Story Defect. Existing ticket: None found. Suggested Jira shape: Story Defect · parent = the owning story SV-8697 · priority Medium · link owning story SV-8697 'relates to' · no Product Area. Re-verify note: ✅ RE-CHECKED 2026-08-19 (v3.8-d0e135e): STILL REPRODUCES — conflicts render amber (text-warning rgb 181,71,8) with the NEW Lucide amber alert-triangle icon on chips + the "9 conflicts" amber pill; NOT red.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Multi-Day Spread Scheduling</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Multi-day spread dialog cannot read the shop's working hours</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>When you drag a job that needs more than one day, the multi-day spread dialog shows the error "Couldn't read this shop's working hours — reopen to try again." (reproduced on three re-opens). This blocks the spread preview: the "{N} shifts / {total}h" summary, the six how-much options with resolved hours, the start-date default, and the weekend-skip distribution. The schedule board itself resolves the same shop's hours fine (7:00–19:00), so the dialog's own hours lookup is failing where the board's succeeds. It does NOT block ordinary single-day shift creation.
 Note for the tester: this may turn out to be a shop-setup precondition on this shop — please have a dev confirm whether the shop needs explicit business hours configured — but on this build the board reads the hours and the dialog does not.</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule on Staging Heavy Duty - 9919.
 2. In the sidebar, find a work order that needs more than one day of work (for example S-9379, about 28.6h remaining).
@@ -749,49 +730,49 @@
 4. Read the multi-day spread dialog.</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>The spread dialog reads the shop's working hours and shows the resolved-hours preview: a "{N} shifts / {total}h" summary, six how-much options with resolved hours, a start date that defaults to the earliest working day, and shifts spread across days skipping weekends only.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.5 (multi-day spread selector + preview); story SV-8691; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>C29979, C29980, C29981, C29982, C29983, C29984, C43802, C43804</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29979  https://shopview.testrail.io/index.php?/cases/view/29980  https://shopview.testrail.io/index.php?/cases/view/29981  https://shopview.testrail.io/index.php?/cases/view/29982  https://shopview.testrail.io/index.php?/cases/view/29983  https://shopview.testrail.io/index.php?/cases/view/29984  https://shopview.testrail.io/index.php?/cases/view/43802  https://shopview.testrail.io/index.php?/cases/view/43804</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Category: CREATE NEW. Recommended action: CREATE NEW Story Defect (first have a dev confirm it is not a shop-config precondition). Existing ticket: None found. Suggested Jira shape: Story Defect · parent = the owning story SV-8691 · priority Medium · link owning story SV-8691 'relates to' · no Product Area. Re-verify note: ✅ RE-CHECKED 2026-08-19 (v3.8-d0e135e): STILL REPRODUCES — dragged S-9379; the spread dialog still shows the red "Couldn't read this shop's working hours — reopen to try again." and Create shifts is disabled. The single-day-preview change did NOT fix hours-read on Heavy Duty 9919.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Drag-and-Drop Scheduling</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>No click-to-arm alternative to dragging a work order</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>There is no way to single-click a sidebar work-order card to "arm" it and then place it on the grid; the only way to schedule is by dragging. The specification's keyboard / accessibility support calls for a click-to-arm alternative. A ticket already captured this (SV-8957) but it is currently closed as Obsolete, and the behaviour still reproduces on the build.</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. In the sidebar, single-click a work-order card (do not drag it).
@@ -799,417 +780,489 @@
 4. Check whether the work order gets scheduled into that cell.</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Clicking a work-order card arms it, and clicking a technician cell then places / schedules it — a click-to-arm alternative to dragging (keyboard / accessibility support).</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §7 (Keyboard support – click-to-arm) / §11 (Accessibility); story SV-8688; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>C29962</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29962</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Category: REOPEN. Recommended action: REOPEN SV-8957 (confirm with Branko that click-to-arm is still required). Existing ticket: SV-8957 (OBSOLETE). Suggested Jira shape: Reopen SV-8957. If it must be refiled as new: Story Defect · parent = the owning story SV-8688 · priority Medium · link owning story SV-8688 'relates to' · no Product Area. Re-verify note: ✅ RE-CHECKED 2026-08-19 (v3.8-d0e135e): STILL REPRODUCES — single-clicking a sidebar card opens the line drill-down (normal behaviour), not "arm"; clicking a cell after schedules nothing (no shift/dialog/toast).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Drag-and-Drop Scheduling</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Month view: dragging a work order onto a day does nothing</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>In Month view, dragging a work order from the sidebar onto a day does not create a shift — nothing happens. The same drag in Week view opens the scope picker and works. A ticket captured this (SV-8870) but it is currently closed as Obsolete, and it still reproduces on the build.
 Note for the tester: the specification does not clearly say whether Month view should accept the drop — this is also a question for Branko to confirm the intended Month-view behaviour.</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule and switch to Month view.
 2. Drag a work order from the sidebar onto a day cell.
 3. Watch whether a shift is created for that day.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Dragging a work order onto a day in Month view creates a shift for that day (the way drag-create works in Week view). Intended Month-view behaviour to be confirmed by Branko.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.1 (drag-and-drop scheduling) / §4.2 (start-time hierarchy); story SV-8688; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>C43555</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/43555</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Category: REOPEN. Recommended action: REOPEN SV-8870 (and confirm with Branko whether Month-view drag-create is intended). Existing ticket: SV-8870 (OBSOLETE). Suggested Jira shape: Reopen SV-8870. If it must be refiled as new: Story Defect · parent = the owning story SV-8688 · priority Medium · link owning story SV-8688 'relates to' · no Product Area. Re-verify note: ✅ RE-CHECKED 2026-08-19 (v3.8-d0e135e): STILL REPRODUCES — Month view reworked (single-line customer+unit chips, today circle, "+N more") but dragging a WO onto a day still does nothing (event count unchanged, no shift/modal/toast).</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Report/Area</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Expected behavior</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>TestRail Case ID(s)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>TestRail Link(s)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>What needs to be done</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Sidebar - Work Order Filters</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Priority filter group is not in the sidebar Filters panel</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>The sidebar Filters panel shows only Assignment and Status — there is no Priority (High / Medium / Low) group. Branko (the Product Owner) ruled on 19 Aug 2026, verbatim "Proceed without it, I'll remove that part from the PRD", so the Priority filter is intentionally removed. The build is correct. NOT a defect — do not file.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Click the sidebar Filters button.
 3. Look at the groups offered.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>The Filters panel offers only two groups: Assignment and Status. Priority is removed per Branko's 19 Aug 2026 ruling; the PRD is to be updated.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Branko (PO) ruling 19 Aug 2026; spec v30 §5.1 (to be updated); story SV-8687; epic SV-8685.</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Branko (PO) ruling 19 Aug 2026; Schedule specification v30 §5.1 (to be updated); story SV-8687; epic SV-8685.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>C29945, C29942</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29945  https://shopview.testrail.io/index.php?/cases/view/29942</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — build is correct (Priority filter intentionally removed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Category: DO NOT FILE. Branko ruled the Priority filter out on 19 Aug 2026 — not a defect, do not file. History: this finding was earlier logged as DEFERRED (feature not found — pending Branko's confirmation on whether Priority filtering was in V1). Branko's 19 Aug 2026 ruling ("Proceed without it, I'll remove that part from the PRD") is the latest authoritative word (Standing Rule 32) and supersedes the deferral. The PRD (spec v30 §5.1) is to be updated to remove Priority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Scope Picker</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Scope picker uses tabs, not a pinned whole-order row (case-wording only)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>The scope picker offers two tabs — "Entire work order" and "Choose lines" — with checkbox line rows, a Select all control and a search box. Some cases describe it as a "pinned whole-order row" with the line rows below. The choice (whole order vs pick individual lines) and the outcome are identical; only the on-screen layout wording differs. This is a test-case wording touch-up, NOT a build defect — do not file.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Drag a multi-line work order onto a technician cell.
 3. Read the scope picker.</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>You can schedule the whole work order or pick individual lines (the build shows this as "Entire work order" / "Choose lines" tabs).</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.3; story SV-8689; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>C29963, C29964, C29965</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29963  https://shopview.testrail.io/index.php?/cases/view/29964  https://shopview.testrail.io/index.php?/cases/view/29965</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — case-wording touch-up only (build behaviour is correct).</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Day View Timeline</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Shift edge-resize not present (feature not built yet)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Dragging a shift's edge to resize it (in 15-minute steps with a live time chip) is not available — the shift block has no resize handles. The feature appears not built yet. Verify with a dev and re-check when it ships. Do not file as a defect.</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule Day view.
 2. Try to drag the top or bottom edge of a shift block.</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Dragging a shift's edge resizes it in 15-minute steps with a live time chip.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.8; stories SV-8694 / SV-9244; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>C30005</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/30005</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — feature not built yet (verify with dev; re-check when it ships).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Day View Timeline</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Day-view zoom control not present (feature not built yet)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>The day view has no zoom control (pixels-per-hour). The feature appears not built yet. Verify with a dev and re-check when it ships. Do not file as a defect.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule Day view.
 2. Look for a zoom control in the day-view toolbar.</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Day view has a zoom control (pixels per hour); blocks and the now-line rescale.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §3.2 / §4.6 / §4.8 / §6; story SV-9244; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>C43812</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/43812</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — feature not built yet (verify with dev; re-check when it ships).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Day View Timeline</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Day-view continuation chevron on a clipped block — could not be verified</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>The continuation-chevron mechanism exists in Week view, but a day-view block clipped by the visible edge could not be produced (no suitable data, and the day-view zoom it relies on is absent), so this could not be confirmed either way. Not a defect. Verify with a dev / re-check when the day-view zoom ships.</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule Day view.
 2. Find a shift clipped by the top or bottom visible edge.
 3. Look for a continuation chevron on it.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>A block clipped by the visible day-view edge shows a continuation chevron.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §3.2 / §4.6 / §4.8 / §6; story SV-9244; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>C43813</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/43813</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — not verifiable / feature dependency not built (verify with dev).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Reassignment and Context Menu</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Assign Work Order from empty-cell menu (automation-held case)</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>The empty-cell menu's first item "Assign Work Order" opens a non-drag scheduling modal — this was confirmed built. This is an automation-held case (owned by the automation side) and its stored body is incomplete. Not a defect — do not file.</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Left-click an empty grid cell.
 3. Choose "Assign Work Order".</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>"Assign Work Order" opens a scheduling modal to schedule an existing work order (feature confirmed built).</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §7 / §4.10 / §14.1; story SV-9242; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>C43811</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/43811</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — automation-held case; feature confirmed built.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Working Hours Settings</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Working Hours settings cases (automation-held)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>The Working Hours settings (business-hours per-day editor, technician custom-hours toggle, inherit shop hours when no custom hours, and Add Hours split ranges) are automation-held cases. Their features rendered / served live on the build; they are owned by the automation side. Not defects — do not file.</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1. Open Settings → Working Hours.
 2. Review the per-day From/To editor and the technician hours toggle.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Business-hours toggle reveals a per-day (Mon-Sun) editor; technician custom-hours toggle off by default; a technician with no custom hours inherits the shop hours; Add Hours appends a removable second range.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.2 (Working Hours); story SV-8699; epic SV-8685.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>C38847, C38848, C38849, C38850</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/38847  https://shopview.testrail.io/index.php?/cases/view/38848  https://shopview.testrail.io/index.php?/cases/view/38849  https://shopview.testrail.io/index.php?/cases/view/38850</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Category: DO NOT FILE. Recommended action: DO NOT FILE — automation-held cases; features confirmed present.</t>
         </is>

</xml_diff>